<commit_message>
Feat: Add dedicated channel deduction cards (實收 vs 已存) for Cash, LINE Pay, Uber Eats, and Foodpanda
</commit_message>
<xml_diff>
--- a/output/本月對帳差額與應收餘額表_202610.xlsx
+++ b/output/本月對帳差額與應收餘額表_202610.xlsx
@@ -580,11 +580,11 @@
     <col width="37.5" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13.5" customWidth="1" min="3" max="3"/>
-    <col width="22.5" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="19.5" customWidth="1" min="7" max="7"/>
-    <col width="67.5" customWidth="1" min="8" max="8"/>
+    <col width="13.5" customWidth="1" min="4" max="4"/>
+    <col width="22.5" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="25.5" customWidth="1" min="7" max="7"/>
+    <col width="73.5" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,22 +605,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>POS 累計營收 (本月權責)</t>
+          <t>① POS 原始額</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>所屬本月實收沖銷</t>
+          <t>② 扣手續費後實收額 (實收)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>手續費發票已沖</t>
+          <t>③ 玉山銀行已存額 (已存)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>目前未收差額 (真實誤差)</t>
+          <t>④ 推算未入帳差額 (實收-已存)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -649,17 +649,17 @@
         <v>186446</v>
       </c>
       <c r="E2" s="3" t="n">
+        <v>186446</v>
+      </c>
+      <c r="F2" s="3" t="n">
         <v>167270</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>19176</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>⏳ 門市尚有 $19,176 現金待存入銀行</t>
+          <t>⏳ 實收現金 $186,446 / 已存現金 $167,270 ➔ 待入帳 $19,176</t>
         </is>
       </c>
     </row>
@@ -683,17 +683,17 @@
         <v>261117</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>228573</v>
+        <v>255075</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>226298</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>32544</v>
+        <v>28777</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>⏳ 連加網路撥款中（預估手續費 $752 / 實撥淨額 $31,792）</t>
+          <t>⏳ 實收LINE Pay $255,075 / 已存 $226,298 ➔ 待入帳 $28,777</t>
         </is>
       </c>
     </row>
@@ -717,17 +717,17 @@
         <v>52523</v>
       </c>
       <c r="E4" s="3" t="n">
+        <v>35190</v>
+      </c>
+      <c r="F4" s="3" t="n">
         <v>28996</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G4" s="3" t="n">
-        <v>23527</v>
+        <v>6194</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>⏳ Uber Eats 結算中（預估抽成發票 $17,333 / 待撥淨額 $6,194）</t>
+          <t>⏳ 實收Uber Eats $35,190 / 已存 $28,996 ➔ 待入帳 $6,194</t>
         </is>
       </c>
     </row>
@@ -751,10 +751,10 @@
         <v>3970</v>
       </c>
       <c r="E5" s="3" t="n">
+        <v>3970</v>
+      </c>
+      <c r="F5" s="3" t="n">
         <v>1870</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>2100</v>
@@ -782,20 +782,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>322417</v>
+        <v>336307</v>
       </c>
       <c r="E6" s="3" t="n">
+        <v>336307</v>
+      </c>
+      <c r="F6" s="3" t="n">
         <v>209228</v>
       </c>
-      <c r="F6" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G6" s="3" t="n">
-        <v>113189</v>
+        <v>127079</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>⏳ 門市尚有 $113,189 現金待存入銀行</t>
+          <t>⏳ 實收現金 $336,307 / 已存現金 $209,228 ➔ 待入帳 $127,079</t>
         </is>
       </c>
     </row>
@@ -816,20 +816,20 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>170122</v>
+        <v>176092</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>95032</v>
+        <v>172017</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>93990</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75090</v>
+        <v>78027</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>⏳ 連加網路撥款中（預估手續費 $1,735 / 實撥淨額 $73,355）</t>
+          <t>⏳ 實收LINE Pay $172,017 / 已存 $93,990 ➔ 待入帳 $78,027</t>
         </is>
       </c>
     </row>
@@ -853,17 +853,17 @@
         <v>16333</v>
       </c>
       <c r="E8" s="3" t="n">
+        <v>11265</v>
+      </c>
+      <c r="F8" s="3" t="n">
         <v>5301</v>
       </c>
-      <c r="F8" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G8" s="3" t="n">
-        <v>11032</v>
+        <v>5964</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>⏳ Uber Eats 結算中（預估抽成發票 $5,390 / 待撥淨額 $5,642）</t>
+          <t>⏳ 實收Uber Eats $11,265 / 已存 $5,301 ➔ 待入帳 $5,964</t>
         </is>
       </c>
     </row>
@@ -884,20 +884,20 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>15596</v>
+        <v>15930</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0</v>
+        <v>10578</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>15596</v>
+        <v>10578</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>⏳ Foodpanda 結算中（預估抽成發票 $5,240 / 待撥淨額 $10,356）</t>
+          <t>⏳ 實收Foodpanda $10,578 / 已存 $0 ➔ 待入帳 $10,578</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3853,6 +3853,54 @@
         </is>
       </c>
       <c r="J12" t="inlineStr">
+        <is>
+          <t>門市正常交班處理中，待總表申報或存款</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>13890</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>❌ 總表U欄空白未填</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 待存入</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>❌ 存摺未見入帳</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>🔴 門市未存 (留店未存)</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>0 天</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>門市正常交班處理中，待總表申報或存款</t>
         </is>
@@ -3961,10 +4009,10 @@
         <v>261117</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>3319</v>
+        <v>6042</v>
       </c>
       <c r="G2" s="12" t="n">
-        <v>158</v>
+        <v>288</v>
       </c>
       <c r="H2" s="12" t="n">
         <v>0</v>
@@ -3976,7 +4024,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>月底核對連加網路 (99024139) 電子發票約 $3,319（含可扣抵進項稅額 $158）</t>
+          <t>月底核對連加網路 (99024139) 電子發票約 $6,042（含可扣抵進項稅額 $288）</t>
         </is>
       </c>
     </row>
@@ -4046,13 +4094,13 @@
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>170122</v>
+        <v>176092</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>2777</v>
+        <v>4075</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>132</v>
+        <v>194</v>
       </c>
       <c r="H4" s="12" t="n">
         <v>0</v>
@@ -4064,7 +4112,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>月底核對連加網路 (99024139) 電子發票約 $2,777（含可扣抵進項稅額 $132）</t>
+          <t>月底核對連加網路 (99024139) 電子發票約 $4,075（含可扣抵進項稅額 $194）</t>
         </is>
       </c>
     </row>
@@ -4086,17 +4134,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>約 33%</t>
+          <t>約 31~33%</t>
         </is>
       </c>
       <c r="E5" s="12" t="n">
         <v>16333</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>5390</v>
+        <v>5068</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="H5" s="12" t="n">
         <v>0</v>
@@ -4108,7 +4156,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>請下載優步 (83118125) 手續費發票約 $5,390 沖銷應收差額（可扣抵稅額 $257）</t>
+          <t>請下載優步 (83118125) 手續費發票約 $5,068 沖銷應收差額（可扣抵稅額 $241）</t>
         </is>
       </c>
     </row>
@@ -4134,13 +4182,13 @@
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>15596</v>
+        <v>15930</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>5240</v>
+        <v>5352</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H6" s="12" t="n">
         <v>0</v>
@@ -4152,7 +4200,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>請下載富胖達 (53075607) 手續費發票約 $5,240 沖銷應收差額（可扣抵稅額 $250）</t>
+          <t>請下載富胖達 (53075607) 手續費發票約 $5,352 沖銷應收差額（可扣抵稅額 $255）</t>
         </is>
       </c>
     </row>

</xml_diff>